<commit_message>
File names for MacOS, F1, accuracy, precision and recall scores and changed readme.md file
</commit_message>
<xml_diff>
--- a/performance_evaluation.xlsx
+++ b/performance_evaluation.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Class Metrics" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion Matrix" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loss per Epoch" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -459,13 +460,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9393939393939394</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9393939393939394</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9393939393939394</v>
+        <v>0.8823529411764706</v>
       </c>
     </row>
     <row r="3">
@@ -475,13 +476,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8</v>
+        <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8</v>
+        <v>0.5555555555555556</v>
       </c>
     </row>
   </sheetData>
@@ -517,10 +518,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -530,10 +531,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -569,7 +570,478 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9069767441860465</v>
+        <v>0.813953488372093</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Epoch</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Train Loss</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Val Loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.6715704202651978</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.6453211903572083</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.6436213850975037</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.6193032264709473</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.6273499131202698</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.5958915948867798</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.6050407886505127</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.5746210813522339</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.5827782154083252</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.5532342195510864</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.5632054209709167</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5322547554969788</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.5402546525001526</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.5120477676391602</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.5187780261039734</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.4928363561630249</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.5089315176010132</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.4751333594322205</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.4985228776931763</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.4590209722518921</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.4844938218593597</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.4448845386505127</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.4731722176074982</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.4325636327266693</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.4565622508525848</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.4219019711017609</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.4587050974369049</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.4124431014060974</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.4451519846916199</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.4038628935813904</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.4475126564502716</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.3959841430187225</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.4432857632637024</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.3882401883602142</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.4312952160835266</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.3804045617580414</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.4315004944801331</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.3721862137317657</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.4132620990276337</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.3638081252574921</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.4106709361076355</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.3555212616920471</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.3874079883098602</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.3476392328739166</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.3728273510932922</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.3398425877094269</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>0.3778283894062042</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.3323823809623718</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.3843465745449066</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.3258050382137299</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0.3803005814552307</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.3203288614749908</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>0.3621543049812317</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.3152017593383789</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0.3485150933265686</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.3102287650108337</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0.3472881317138672</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.3050626218318939</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>0.3528615832328796</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.3002362549304962</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>0.339249849319458</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.295564591884613</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>0.3337916731834412</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.2907191216945648</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>0.3356787860393524</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.2857457995414734</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>0.3279911577701569</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.281109631061554</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>0.3238618075847626</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.2769296169281006</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>0.3167205154895782</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.2733596861362457</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>0.3136237263679504</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.2703306972980499</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>0.3298770189285278</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.2679539322853088</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>0.3098456561565399</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.2660715579986572</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>0.3076216876506805</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.2642519176006317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>